<commit_message>
Dizayn to'liq zumrad va neon yashil (Emerald Green) ranglar bilan yangilandi
</commit_message>
<xml_diff>
--- a/exports/namuna_kontaktlar.xlsx
+++ b/exports/namuna_kontaktlar.xlsx
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="003B82F6"/>
-        <bgColor rgb="003B82F6"/>
+        <fgColor rgb="0010B981"/>
+        <bgColor rgb="0010B981"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>